<commit_message>
Actualización de la documentación FASE I Business Undertanding posterior a la reunión semanal 9/9/2026
</commit_message>
<xml_diff>
--- a/01_Business_Understanding/Project_Charter.xlsx
+++ b/01_Business_Understanding/Project_Charter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gplaneta-my.sharepoint.com/personal/umgz4a_psoplaneta_com/Documents/DATA/Analytics Projects/Product_Analytics/01_Business_Understanding/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="8_{2808834A-88FA-488B-A429-3D647F25CCEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{014E6DFA-6E41-4109-B66E-2D0B085214A0}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="8_{2808834A-88FA-488B-A429-3D647F25CCEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78048106-F342-4B21-B489-986EBB613A0E}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -259,22 +259,23 @@
     <t>Programas con todos sus programas activos en ofertas comparables válidas</t>
   </si>
   <si>
+    <t>Diseñar, validar y publicar un dashboard ejecutivo en Power BI que consolide los programas de la institución, o aquellos que se quieran proponer para el nuevo portafolio, sus comparables directos, precios y diferenciales verificables, e histórico de matrículas SNIES de los últimos cinco años disponibles; permitiendo identificar competencia directa y soportar decisiones de precio, propuesta de valor, comportamiento del mercado, portafolio y captación.</t>
+  </si>
+  <si>
+    <t>Proyecto dashboard de Inteligencia Competitiva de Precios y Demanda</t>
+  </si>
+  <si>
+    <t>01_Business_Understanding</t>
+  </si>
+  <si>
     <t>INCLUYE
 • Inventario y homologación de programas y ofertas comparables.
 • Criterios y puntaje de competencia directa: afinidad académica, modalidad, ubicación/segmento, precio, demanda y diferenciales.
 • Precios normalizados, descuentos y vigencia; fuentes de cliente oculto. 
 • Histórico SNIES de los últimos 5 años disponibles.
 • Modelo de datos y dashboard PBI: resumen ejecutivo, comparado por programa, mapa competitivo precio–valor, tendencias de matrícula y trazabilidad.
-• Publicación, perfiles de acceso, documentación y capacitación.</t>
-  </si>
-  <si>
-    <t>Diseñar, validar y publicar un dashboard ejecutivo en Power BI que consolide los programas de la institución, o aquellos que se quieran proponer para el nuevo portafolio, sus comparables directos, precios y diferenciales verificables, e histórico de matrículas SNIES de los últimos cinco años disponibles; permitiendo identificar competencia directa y soportar decisiones de precio, propuesta de valor, comportamiento del mercado, portafolio y captación.</t>
-  </si>
-  <si>
-    <t>Proyecto dashboard de Inteligencia Competitiva de Precios y Demanda</t>
-  </si>
-  <si>
-    <t>01_Business_Understanding</t>
+• Publicación, perfiles de acceso, documentación y capacitación.
+Alcance del proyecto 2020 - 2026</t>
   </si>
 </sst>
 </file>
@@ -751,6 +752,42 @@
     </xf>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="6" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -760,6 +797,48 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -799,89 +878,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -950,10 +951,6 @@
     <xdr:clientData/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5015,60 +5012,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="11" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="36" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="26"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="38"/>
     </row>
     <row r="2" spans="1:10" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="30"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="55" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="56"/>
     </row>
     <row r="3" spans="1:10" ht="11" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="26"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="37"/>
+      <c r="H3" s="37"/>
+      <c r="I3" s="38"/>
     </row>
     <row r="4" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="66" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="43"/>
-      <c r="C4" s="38" t="s">
+      <c r="B4" s="67"/>
+      <c r="C4" s="64" t="s">
         <v>61</v>
       </c>
-      <c r="D4" s="38"/>
-      <c r="E4" s="38"/>
-      <c r="F4" s="38"/>
-      <c r="G4" s="38"/>
-      <c r="H4" s="38"/>
-      <c r="I4" s="39"/>
+      <c r="D4" s="64"/>
+      <c r="E4" s="64"/>
+      <c r="F4" s="64"/>
+      <c r="G4" s="64"/>
+      <c r="H4" s="64"/>
+      <c r="I4" s="65"/>
       <c r="J4" s="2"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -5076,68 +5073,68 @@
         <v>30</v>
       </c>
       <c r="B5" s="41"/>
-      <c r="C5" s="35" t="s">
+      <c r="C5" s="61" t="s">
         <v>62</v>
       </c>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="36"/>
-      <c r="I5" s="37"/>
+      <c r="D5" s="62"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="62"/>
+      <c r="G5" s="62"/>
+      <c r="H5" s="62"/>
+      <c r="I5" s="63"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="40"/>
       <c r="B6" s="41"/>
-      <c r="C6" s="36"/>
-      <c r="D6" s="36"/>
-      <c r="E6" s="36"/>
-      <c r="F6" s="36"/>
-      <c r="G6" s="36"/>
-      <c r="H6" s="36"/>
-      <c r="I6" s="37"/>
+      <c r="C6" s="62"/>
+      <c r="D6" s="62"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
+      <c r="G6" s="62"/>
+      <c r="H6" s="62"/>
+      <c r="I6" s="63"/>
     </row>
     <row r="7" spans="1:10" ht="86.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="40"/>
       <c r="B7" s="41"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="37"/>
+      <c r="C7" s="62"/>
+      <c r="D7" s="62"/>
+      <c r="E7" s="62"/>
+      <c r="F7" s="62"/>
+      <c r="G7" s="62"/>
+      <c r="H7" s="62"/>
+      <c r="I7" s="63"/>
       <c r="J7" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="57" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="32"/>
-      <c r="C8" s="33" t="s">
+      <c r="B8" s="58"/>
+      <c r="C8" s="59" t="s">
         <v>52</v>
       </c>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="34"/>
+      <c r="D8" s="59"/>
+      <c r="E8" s="59"/>
+      <c r="F8" s="59"/>
+      <c r="G8" s="59"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="60"/>
     </row>
     <row r="9" spans="1:10" ht="11" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="24" t="s">
+      <c r="A9" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="25"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="26"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="38"/>
     </row>
     <row r="10" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="46" t="s">
@@ -5145,7 +5142,7 @@
       </c>
       <c r="B10" s="47"/>
       <c r="C10" s="48" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D10" s="48"/>
       <c r="E10" s="48"/>
@@ -5176,13 +5173,13 @@
     <row r="12" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="51"/>
       <c r="B12" s="52"/>
-      <c r="C12" s="44" t="s">
+      <c r="C12" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="D12" s="44"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="44"/>
-      <c r="G12" s="44"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
       <c r="H12" s="22">
         <v>0</v>
       </c>
@@ -5193,13 +5190,13 @@
     <row r="13" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="51"/>
       <c r="B13" s="52"/>
-      <c r="C13" s="44" t="s">
+      <c r="C13" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="44"/>
-      <c r="E13" s="44"/>
-      <c r="F13" s="44"/>
-      <c r="G13" s="44"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
       <c r="H13" s="22">
         <v>0</v>
       </c>
@@ -5210,13 +5207,13 @@
     <row r="14" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="51"/>
       <c r="B14" s="52"/>
-      <c r="C14" s="44" t="s">
+      <c r="C14" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="44"/>
-      <c r="G14" s="44"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
       <c r="H14" s="15">
         <v>0</v>
       </c>
@@ -5227,13 +5224,13 @@
     <row r="15" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="51"/>
       <c r="B15" s="52"/>
-      <c r="C15" s="44" t="s">
+      <c r="C15" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="D15" s="44"/>
-      <c r="E15" s="44"/>
-      <c r="F15" s="44"/>
-      <c r="G15" s="44"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
       <c r="H15" s="15">
         <v>0</v>
       </c>
@@ -5246,107 +5243,107 @@
         <v>39</v>
       </c>
       <c r="B16" s="41"/>
-      <c r="C16" s="44" t="s">
-        <v>64</v>
-      </c>
-      <c r="D16" s="44"/>
-      <c r="E16" s="44"/>
+      <c r="C16" s="34" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16" s="34"/>
+      <c r="E16" s="34"/>
       <c r="F16" s="41" t="s">
         <v>40</v>
       </c>
       <c r="G16" s="41"/>
-      <c r="H16" s="44" t="s">
+      <c r="H16" s="34" t="s">
         <v>57</v>
       </c>
-      <c r="I16" s="45"/>
+      <c r="I16" s="35"/>
     </row>
     <row r="17" spans="1:9" ht="179.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="40"/>
       <c r="B17" s="41"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="44"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
       <c r="F17" s="41"/>
       <c r="G17" s="41"/>
-      <c r="H17" s="44"/>
-      <c r="I17" s="45"/>
+      <c r="H17" s="34"/>
+      <c r="I17" s="35"/>
     </row>
     <row r="18" spans="1:9" ht="30.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="40" t="s">
         <v>41</v>
       </c>
       <c r="B18" s="41"/>
-      <c r="C18" s="44" t="s">
+      <c r="C18" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="D18" s="44"/>
-      <c r="E18" s="44"/>
-      <c r="F18" s="44"/>
-      <c r="G18" s="44"/>
-      <c r="H18" s="44"/>
-      <c r="I18" s="45"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
+      <c r="I18" s="35"/>
     </row>
     <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="40" t="s">
         <v>42</v>
       </c>
       <c r="B19" s="41"/>
-      <c r="C19" s="61" t="s">
+      <c r="C19" s="44" t="s">
         <v>36</v>
       </c>
-      <c r="D19" s="61"/>
-      <c r="E19" s="61"/>
-      <c r="F19" s="61"/>
-      <c r="G19" s="61" t="s">
+      <c r="D19" s="44"/>
+      <c r="E19" s="44"/>
+      <c r="F19" s="44"/>
+      <c r="G19" s="44" t="s">
         <v>43</v>
       </c>
-      <c r="H19" s="61"/>
-      <c r="I19" s="62"/>
+      <c r="H19" s="44"/>
+      <c r="I19" s="45"/>
     </row>
     <row r="20" spans="1:9" ht="11" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="59"/>
-      <c r="B20" s="60"/>
-      <c r="C20" s="53" t="s">
+      <c r="A20" s="42"/>
+      <c r="B20" s="43"/>
+      <c r="C20" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="D20" s="53"/>
-      <c r="E20" s="53"/>
-      <c r="F20" s="53"/>
-      <c r="G20" s="53" t="s">
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="H20" s="53"/>
-      <c r="I20" s="54"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="33"/>
     </row>
     <row r="21" spans="1:9" ht="11" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="24" t="s">
+      <c r="A21" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="25"/>
-      <c r="I21" s="26"/>
+      <c r="B21" s="37"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="37"/>
+      <c r="I21" s="38"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="57" t="s">
+      <c r="A22" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="58"/>
+      <c r="B22" s="31"/>
       <c r="C22" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D22" s="58" t="s">
+      <c r="D22" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="E22" s="58"/>
-      <c r="F22" s="58" t="s">
+      <c r="E22" s="31"/>
+      <c r="F22" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="G22" s="58"/>
+      <c r="G22" s="31"/>
       <c r="H22" s="18" t="s">
         <v>48</v>
       </c>
@@ -5355,128 +5352,128 @@
       </c>
     </row>
     <row r="23" spans="1:9" s="11" customFormat="1" ht="49.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="55" t="s">
+      <c r="A23" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B23" s="56"/>
+      <c r="B23" s="28"/>
       <c r="C23" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D23" s="63" t="s">
+      <c r="D23" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="E23" s="63"/>
-      <c r="F23" s="63" t="s">
+      <c r="E23" s="25"/>
+      <c r="F23" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="G23" s="63"/>
-      <c r="H23" s="67" t="s">
-        <v>67</v>
+      <c r="G23" s="25"/>
+      <c r="H23" s="24" t="s">
+        <v>66</v>
       </c>
       <c r="I23" s="10" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="24" spans="1:9" s="11" customFormat="1" ht="64" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="55" t="s">
+      <c r="A24" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="56"/>
+      <c r="B24" s="28"/>
       <c r="C24" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D24" s="63" t="s">
+      <c r="D24" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="E24" s="63"/>
-      <c r="F24" s="63" t="s">
+      <c r="E24" s="25"/>
+      <c r="F24" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="G24" s="63"/>
+      <c r="G24" s="25"/>
       <c r="H24" s="9"/>
       <c r="I24" s="10" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="25" spans="1:9" s="11" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="55" t="s">
+      <c r="A25" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B25" s="56"/>
+      <c r="B25" s="28"/>
       <c r="C25" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D25" s="63" t="s">
+      <c r="D25" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="E25" s="63"/>
-      <c r="F25" s="63" t="s">
+      <c r="E25" s="25"/>
+      <c r="F25" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="G25" s="63"/>
+      <c r="G25" s="25"/>
       <c r="H25" s="9"/>
       <c r="I25" s="10" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="26" spans="1:9" s="11" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="55" t="s">
+      <c r="A26" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="B26" s="56"/>
+      <c r="B26" s="28"/>
       <c r="C26" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D26" s="63" t="s">
+      <c r="D26" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="E26" s="63"/>
-      <c r="F26" s="63" t="s">
+      <c r="E26" s="25"/>
+      <c r="F26" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="G26" s="63"/>
+      <c r="G26" s="25"/>
       <c r="H26" s="9"/>
       <c r="I26" s="10" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="27" spans="1:9" s="11" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="55" t="s">
+      <c r="A27" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="56"/>
+      <c r="B27" s="28"/>
       <c r="C27" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D27" s="63" t="s">
+      <c r="D27" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="E27" s="63"/>
-      <c r="F27" s="63" t="s">
+      <c r="E27" s="25"/>
+      <c r="F27" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="G27" s="63"/>
+      <c r="G27" s="25"/>
       <c r="H27" s="9"/>
       <c r="I27" s="10" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="28" spans="1:9" s="11" customFormat="1" ht="44.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="65" t="s">
+      <c r="A28" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="B28" s="66"/>
+      <c r="B28" s="30"/>
       <c r="C28" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D28" s="64" t="s">
+      <c r="D28" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="E28" s="64"/>
-      <c r="F28" s="64" t="s">
+      <c r="E28" s="26"/>
+      <c r="F28" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="G28" s="64"/>
+      <c r="G28" s="26"/>
       <c r="H28" s="13"/>
       <c r="I28" s="14" t="s">
         <v>59</v>
@@ -5484,18 +5481,30 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="C2:I2"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:I8"/>
+    <mergeCell ref="C5:I7"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="A5:B7"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A16:B17"/>
+    <mergeCell ref="C16:E17"/>
+    <mergeCell ref="F16:G17"/>
+    <mergeCell ref="H16:I17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:I10"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="A11:B15"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="C14:G14"/>
+    <mergeCell ref="C15:G15"/>
     <mergeCell ref="C20:F20"/>
     <mergeCell ref="G20:I20"/>
     <mergeCell ref="C18:I18"/>
@@ -5512,30 +5521,18 @@
     <mergeCell ref="F23:G23"/>
     <mergeCell ref="F24:G24"/>
     <mergeCell ref="F25:G25"/>
-    <mergeCell ref="A9:I9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C10:I10"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="A11:B15"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="C14:G14"/>
-    <mergeCell ref="C15:G15"/>
-    <mergeCell ref="A16:B17"/>
-    <mergeCell ref="C16:E17"/>
-    <mergeCell ref="F16:G17"/>
-    <mergeCell ref="H16:I17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="C2:I2"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:I8"/>
-    <mergeCell ref="C5:I7"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="A5:B7"/>
-    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H23" r:id="rId1" xr:uid="{4A9A01C2-595E-46B3-82AB-AA30192D9F42}"/>
@@ -5546,6 +5543,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b593fc4c-2af5-4cc2-b6db-90e9851bf100">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="46c87129-2922-41e0-9915-4492c14b85cf" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101009200D15403517347BFCC7BEE816B18F5" ma:contentTypeVersion="14" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a0825bdce9e1781b945402c59db5edc8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="299da364-5bd6-4856-b54f-296f95f3dc71" xmlns:ns3="b593fc4c-2af5-4cc2-b6db-90e9851bf100" xmlns:ns4="7fe59f34-55a4-4ccc-9a2c-36cfcecf2037" xmlns:ns5="46c87129-2922-41e0-9915-4492c14b85cf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="02cdc2cddc775292ee59ef2ed547c7df" ns2:_="" ns3:_="" ns4:_="" ns5:_="">
     <xsd:import namespace="299da364-5bd6-4856-b54f-296f95f3dc71"/>
@@ -5786,17 +5794,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b593fc4c-2af5-4cc2-b6db-90e9851bf100">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="46c87129-2922-41e0-9915-4492c14b85cf" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -5807,6 +5804,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2C3076F-6400-4B81-A360-51EB9A96E88E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b593fc4c-2af5-4cc2-b6db-90e9851bf100"/>
+    <ds:schemaRef ds:uri="46c87129-2922-41e0-9915-4492c14b85cf"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6920F35-F84F-4729-89D9-C286674B0283}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5827,17 +5835,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2C3076F-6400-4B81-A360-51EB9A96E88E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b593fc4c-2af5-4cc2-b6db-90e9851bf100"/>
-    <ds:schemaRef ds:uri="46c87129-2922-41e0-9915-4492c14b85cf"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DB84459-FF79-406B-9DBE-8152F6CED2CC}">
   <ds:schemaRefs>

</xml_diff>